<commit_message>
Updated ITA model - 2025-09-07 18:48
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C79CEB39-11C3-417F-92F4-CBAC55936ABE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4B8115A0-937D-4714-8256-FD7D6606F4C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7796,7 +7796,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F945F4DC-6461-480E-B139-B512F79E4095}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{535A71C7-DDB3-44A4-BEF3-471BE1CE6331}">
   <dimension ref="B9:N50"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9372,7 +9372,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F798780-7963-4D2E-A138-7EA392735E10}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6F414BC-A8B6-4AD0-9AC2-3A617E989096}">
   <dimension ref="B9:AB172"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -21314,7 +21314,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4136A2E-5B4E-4CA1-BD11-3CBE85D22ADA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8032EF8C-1FA6-45C7-841B-0266961AB77D}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA model - 2025-09-07 19:10
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4B8115A0-937D-4714-8256-FD7D6606F4C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{97A055C2-E6B7-49E7-9895-FE26BC7A1498}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7796,7 +7796,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{535A71C7-DDB3-44A4-BEF3-471BE1CE6331}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5CD4E9D-01E2-44C5-9E07-5170D1FD901F}">
   <dimension ref="B9:N50"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9372,7 +9372,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6F414BC-A8B6-4AD0-9AC2-3A617E989096}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54578B1C-2A48-4D65-9949-83DB11632B55}">
   <dimension ref="B9:AB172"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -21314,7 +21314,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8032EF8C-1FA6-45C7-841B-0266961AB77D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99B04B7C-0243-4E8A-8582-394465F09F63}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA model - 2025-09-08 00:48
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{97A055C2-E6B7-49E7-9895-FE26BC7A1498}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0AF61530-54E9-4670-AF7F-26D031995271}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7796,7 +7796,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5CD4E9D-01E2-44C5-9E07-5170D1FD901F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEE89816-0DDB-4A66-AB5F-FBB5D461DF34}">
   <dimension ref="B9:N50"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9372,7 +9372,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54578B1C-2A48-4D65-9949-83DB11632B55}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE9F5C3C-D685-4A46-BCDE-1C5015252609}">
   <dimension ref="B9:AB172"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -21314,7 +21314,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99B04B7C-0243-4E8A-8582-394465F09F63}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97B2FC12-338A-42A9-950C-083D776F31AF}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA model - 2025-09-11 18:55
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B661F2B3-861D-4EFC-9586-322ACFEDF49A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8EDAB741-F939-4CC8-94D9-2BA4F3DEC19A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4008" uniqueCount="937">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4010" uniqueCount="937">
   <si>
     <t>~FI_Process</t>
   </si>
@@ -4478,7 +4478,9 @@
       <c r="F8" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="1"/>
+      <c r="G8" t="s">
+        <v>14</v>
+      </c>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
       <c r="J8" s="1" t="str">
@@ -4514,7 +4516,9 @@
       <c r="F9" t="s">
         <v>10</v>
       </c>
-      <c r="G9" s="1"/>
+      <c r="G9" t="s">
+        <v>14</v>
+      </c>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
       <c r="K9" s="1"/>
@@ -7796,7 +7800,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A61423C4-5CFB-4BFA-AE3D-4AAF86248DD1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B25634C-2603-4E95-AFFD-C3D4ACDE4FCE}">
   <dimension ref="B9:N50"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9372,7 +9376,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C0CC65C-E8D3-4E9D-95CC-48AA0DA6A8C1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{161A821A-5581-4AD8-B47F-8B101878B4A5}">
   <dimension ref="B9:AB172"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -21314,7 +21318,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55A855E2-40DE-4A3F-A0EC-0028635FA9E1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DB4C948-6C77-47D7-89C0-0CF3E8E47619}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA model - 2025-09-13 15:17
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8EDAB741-F939-4CC8-94D9-2BA4F3DEC19A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AEE6F11A-535D-40B2-8CD1-E8B627FEB325}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7800,7 +7800,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B25634C-2603-4E95-AFFD-C3D4ACDE4FCE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10F53C81-D1C9-445E-AE69-1BAE6209A4FC}">
   <dimension ref="B9:N50"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9376,7 +9376,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{161A821A-5581-4AD8-B47F-8B101878B4A5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{408D71EE-D7FC-4382-BD1F-5F95F4D27495}">
   <dimension ref="B9:AB172"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -21318,7 +21318,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DB4C948-6C77-47D7-89C0-0CF3E8E47619}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D299C06F-01AD-40CE-90FB-48FB0B4D5260}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA model - 2025-09-13 16:26
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AEE6F11A-535D-40B2-8CD1-E8B627FEB325}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{444C6A8B-A731-485F-9B13-5E4E160BBA7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7800,7 +7800,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10F53C81-D1C9-445E-AE69-1BAE6209A4FC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8401CED8-5767-412E-AC5C-B83BDE74EB69}">
   <dimension ref="B9:N50"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9376,7 +9376,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{408D71EE-D7FC-4382-BD1F-5F95F4D27495}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{036C8E3B-E0F2-4996-BAB8-C97D22769EF3}">
   <dimension ref="B9:AB172"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -21318,7 +21318,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D299C06F-01AD-40CE-90FB-48FB0B4D5260}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC680C18-4A4B-49F8-88E4-F3E9B23A8DFD}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA model - 2025-09-14 12:57
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{444C6A8B-A731-485F-9B13-5E4E160BBA7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{67720356-68E5-4D07-92E7-D0AA15EBCC12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7800,7 +7800,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8401CED8-5767-412E-AC5C-B83BDE74EB69}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C56D50E6-0D10-493A-877F-C7BDFED6843F}">
   <dimension ref="B9:N50"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9376,7 +9376,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{036C8E3B-E0F2-4996-BAB8-C97D22769EF3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D764C90D-33F1-47E0-95F3-8138E964B8FF}">
   <dimension ref="B9:AB172"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -21318,7 +21318,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC680C18-4A4B-49F8-88E4-F3E9B23A8DFD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C52733C6-A850-4C56-B923-44EF58869B7A}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA model - 2025-09-14 13:01
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{67720356-68E5-4D07-92E7-D0AA15EBCC12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A3F5B2AB-7ADE-486E-BD3D-35829BA843F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7800,7 +7800,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C56D50E6-0D10-493A-877F-C7BDFED6843F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B3C8ECB-F941-4AC5-A2CC-CF7B8BD87E99}">
   <dimension ref="B9:N50"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9376,7 +9376,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D764C90D-33F1-47E0-95F3-8138E964B8FF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58E36B8F-8782-4775-9F99-94590F617DE4}">
   <dimension ref="B9:AB172"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -21318,7 +21318,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C52733C6-A850-4C56-B923-44EF58869B7A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40BB2464-2769-4EDF-BC03-024EF3A42093}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA model - 2025-09-14 13:04
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A3F5B2AB-7ADE-486E-BD3D-35829BA843F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A0EA7714-9EFF-46DA-8496-E475447875FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7800,7 +7800,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B3C8ECB-F941-4AC5-A2CC-CF7B8BD87E99}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C789FDA1-21CE-4730-ADA0-DC42CFD28EC9}">
   <dimension ref="B9:N50"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9376,7 +9376,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58E36B8F-8782-4775-9F99-94590F617DE4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C49CD672-47E5-4A7A-B9F0-A7E778EFAFE6}">
   <dimension ref="B9:AB172"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -21318,7 +21318,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40BB2464-2769-4EDF-BC03-024EF3A42093}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3BD1BDA-0930-43CE-ACCC-2B0BCC2B2988}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA model - 2025-09-14 13:18
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A0EA7714-9EFF-46DA-8496-E475447875FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4B821FA3-C3E5-4628-97FF-8E1B12524B93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7800,7 +7800,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C789FDA1-21CE-4730-ADA0-DC42CFD28EC9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA9EDF41-37E3-4CF2-B311-52F405C06AB5}">
   <dimension ref="B9:N50"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9376,7 +9376,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C49CD672-47E5-4A7A-B9F0-A7E778EFAFE6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12DE61B3-A1E1-4635-8B25-6D9EA10B9C72}">
   <dimension ref="B9:AB172"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -21318,7 +21318,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3BD1BDA-0930-43CE-ACCC-2B0BCC2B2988}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{894BA582-9E81-4AD1-A523-1C8B9CB48F29}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA model - 2025-09-14 13:29
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4B821FA3-C3E5-4628-97FF-8E1B12524B93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E6C238D6-BC46-4F3A-B83F-BF78C7DE5281}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7800,7 +7800,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA9EDF41-37E3-4CF2-B311-52F405C06AB5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA76C70E-2DE9-46E3-8DD8-B6EB456733F7}">
   <dimension ref="B9:N50"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9376,7 +9376,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12DE61B3-A1E1-4635-8B25-6D9EA10B9C72}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A98200BF-E0DC-4BCF-8219-D78A29556B65}">
   <dimension ref="B9:AB172"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -21318,7 +21318,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{894BA582-9E81-4AD1-A523-1C8B9CB48F29}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4ACB1D4D-A02B-42B5-A45C-CDEFDB97A3AC}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA model - 2025-09-14 17:56
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E6C238D6-BC46-4F3A-B83F-BF78C7DE5281}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A6CB32CD-3E4C-46D8-B509-CB88DA1BF47A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7800,7 +7800,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA76C70E-2DE9-46E3-8DD8-B6EB456733F7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87338818-4BE2-4E4B-988C-8109526D603E}">
   <dimension ref="B9:N50"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9376,7 +9376,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A98200BF-E0DC-4BCF-8219-D78A29556B65}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63BC8720-F713-4C67-A36B-21824F7EC03F}">
   <dimension ref="B9:AB172"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -21318,7 +21318,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4ACB1D4D-A02B-42B5-A45C-CDEFDB97A3AC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3FB6245-ED28-4D6F-BED0-F116AD59ABF7}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA model - 2025-09-17 00:29
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6BB03A8D-259A-4775-8093-D7C74DC34750}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4FE11156-6AAA-4E7F-A5ED-5C7C5CCCAA7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6186,7 +6186,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E8888BE-6C99-4F02-9ED7-5FD54C15DA75}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9E9C4AB-A26C-4D00-B016-8A940A10ED3E}">
   <dimension ref="B9:M34"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -7079,7 +7079,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E17D573-917B-4284-B4C6-972A80CC0D48}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{026C1A0C-80D1-4975-AD58-BC67870AFEDF}">
   <dimension ref="B9:Z29"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -8463,7 +8463,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41E5E5B0-0EAF-4C89-864D-DFEEF39709ED}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8C50719-33A8-449C-91F4-3FBA20552F7A}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA model - 2025-09-17 00:49
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4FE11156-6AAA-4E7F-A5ED-5C7C5CCCAA7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1DF9AF6D-4739-4009-A8E9-C53DFD5B35FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="735" yWindow="735" windowWidth="21600" windowHeight="12682" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="misc" sheetId="7" r:id="rId1"/>
@@ -6186,7 +6186,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9E9C4AB-A26C-4D00-B016-8A940A10ED3E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50D34FB4-0CEE-4A8C-AD48-2038A5041932}">
   <dimension ref="B9:M34"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -7079,7 +7079,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{026C1A0C-80D1-4975-AD58-BC67870AFEDF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F3C3EDC-C8B1-4325-9BCA-C3C0D4F45D9A}">
   <dimension ref="B9:Z29"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -8463,7 +8463,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8C50719-33A8-449C-91F4-3FBA20552F7A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B90F391E-6A9E-4214-B2BE-D817628AF288}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA model - 2025-09-17 02:00
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1DF9AF6D-4739-4009-A8E9-C53DFD5B35FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FABB4715-6ACB-46EB-9E58-C46181B3E7DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="735" yWindow="735" windowWidth="21600" windowHeight="12682" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="368" yWindow="368" windowWidth="21599" windowHeight="12682" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="misc" sheetId="7" r:id="rId1"/>
@@ -1084,115 +1084,115 @@
     <t>e_wof_001</t>
   </si>
   <si>
-    <t>offshore wind resource in cluster 1</t>
+    <t>wind offshore resource in cluster 1</t>
   </si>
   <si>
     <t>e_wof_002</t>
   </si>
   <si>
-    <t>offshore wind resource in cluster 2</t>
+    <t>wind offshore resource in cluster 2</t>
   </si>
   <si>
     <t>e_wof_003</t>
   </si>
   <si>
-    <t>offshore wind resource in cluster 3</t>
+    <t>wind offshore resource in cluster 3</t>
   </si>
   <si>
     <t>e_wof_004</t>
   </si>
   <si>
-    <t>offshore wind resource in cluster 4</t>
+    <t>wind offshore resource in cluster 4</t>
   </si>
   <si>
     <t>e_wof_005</t>
   </si>
   <si>
-    <t>offshore wind resource in cluster 5</t>
+    <t>wind offshore resource in cluster 5</t>
   </si>
   <si>
     <t>e_wof_006</t>
   </si>
   <si>
-    <t>offshore wind resource in cluster 6</t>
+    <t>wind offshore resource in cluster 6</t>
   </si>
   <si>
     <t>e_wof_007</t>
   </si>
   <si>
-    <t>offshore wind resource in cluster 7</t>
+    <t>wind offshore resource in cluster 7</t>
   </si>
   <si>
     <t>e_wof_008</t>
   </si>
   <si>
-    <t>offshore wind resource in cluster 8</t>
+    <t>wind offshore resource in cluster 8</t>
   </si>
   <si>
     <t>e_wof_009</t>
   </si>
   <si>
-    <t>offshore wind resource in cluster 9</t>
+    <t>wind offshore resource in cluster 9</t>
   </si>
   <si>
     <t>e_wof_010</t>
   </si>
   <si>
-    <t>offshore wind resource in cluster 10</t>
+    <t>wind offshore resource in cluster 10</t>
   </si>
   <si>
     <t>e_wof_011</t>
   </si>
   <si>
-    <t>offshore wind resource in cluster 11</t>
+    <t>wind offshore resource in cluster 11</t>
   </si>
   <si>
     <t>e_wof_012</t>
   </si>
   <si>
-    <t>offshore wind resource in cluster 12</t>
+    <t>wind offshore resource in cluster 12</t>
   </si>
   <si>
     <t>e_wof_013</t>
   </si>
   <si>
-    <t>offshore wind resource in cluster 13</t>
+    <t>wind offshore resource in cluster 13</t>
   </si>
   <si>
     <t>e_wof_014</t>
   </si>
   <si>
-    <t>offshore wind resource in cluster 14</t>
+    <t>wind offshore resource in cluster 14</t>
   </si>
   <si>
     <t>e_wof_015</t>
   </si>
   <si>
-    <t>offshore wind resource in cluster 15</t>
+    <t>wind offshore resource in cluster 15</t>
   </si>
   <si>
     <t>e_wof_016</t>
   </si>
   <si>
-    <t>offshore wind resource in cluster 16</t>
+    <t>wind offshore resource in cluster 16</t>
   </si>
   <si>
     <t>e_wof_017</t>
   </si>
   <si>
-    <t>offshore wind resource in cluster 17</t>
+    <t>wind offshore resource in cluster 17</t>
   </si>
   <si>
     <t>e_wof_018</t>
   </si>
   <si>
-    <t>offshore wind resource in cluster 18</t>
+    <t>wind offshore resource in cluster 18</t>
   </si>
   <si>
     <t>e_wof_019</t>
   </si>
   <si>
-    <t>offshore wind resource in cluster 19</t>
+    <t>wind offshore resource in cluster 19</t>
   </si>
   <si>
     <t>elc_wof_001</t>
@@ -6186,7 +6186,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50D34FB4-0CEE-4A8C-AD48-2038A5041932}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9223088-4856-4BAF-941C-BB59CDA416A2}">
   <dimension ref="B9:M34"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -7079,7 +7079,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F3C3EDC-C8B1-4325-9BCA-C3C0D4F45D9A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7312D715-8B93-41D9-A5C4-8F03E52428E5}">
   <dimension ref="B9:Z29"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -8463,7 +8463,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B90F391E-6A9E-4214-B2BE-D817628AF288}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58A37DE2-93D6-40E8-9544-296B49811748}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA model - 2025-09-17 09:29
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FABB4715-6ACB-46EB-9E58-C46181B3E7DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B733CC57-A96D-4FC1-91D7-131FE8E967FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="368" yWindow="368" windowWidth="21599" windowHeight="12682" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3308" yWindow="3308" windowWidth="21600" windowHeight="12682" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="misc" sheetId="7" r:id="rId1"/>
@@ -6186,7 +6186,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9223088-4856-4BAF-941C-BB59CDA416A2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74DF7FAD-AD3F-4587-A19A-8E82EAFCD442}">
   <dimension ref="B9:M34"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -7079,7 +7079,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7312D715-8B93-41D9-A5C4-8F03E52428E5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{073B4C54-CB90-4706-86A3-0F1CA0120467}">
   <dimension ref="B9:Z29"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -8463,7 +8463,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58A37DE2-93D6-40E8-9544-296B49811748}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A303DFC-8E26-40F9-A8C3-C850F186FDD7}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA model - 2025-12-12 15:41
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_ITA/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{48E2839C-DDF9-4DE0-ADC2-C865799D4278}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CEB0862E-B885-4185-8E20-36395C0D1BD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1283" uniqueCount="389">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1284" uniqueCount="391">
   <si>
     <t>~FI_Process</t>
   </si>
@@ -618,6 +618,9 @@
     <t>wnid offshore potential</t>
   </si>
   <si>
+    <t>ELC_BatIn</t>
+  </si>
+  <si>
     <t>~fi_process</t>
   </si>
   <si>
@@ -1294,6 +1297,9 @@
   </si>
   <si>
     <t>yes</t>
+  </si>
+  <si>
+    <t>e_IT10-380,e_IT156-380,e_IT157-380,e_IT158-380,e_IT159-380,e_IT21-380,e_IT42-380,e_IT7-380,e_IT8-380,e_IT9-380,e_IT90-400,e_IT93-380,e_w100113593-380,e_w100407576-380,e_w103381531-380,e_w103653592-380,e_w105757794-380,e_w109588422-380,e_w109756016-380,e_w109993642-380,e_w109997676-380,e_w110138220-380,e_w1103579629-380,e_w110660048-380,e_w1117128898-380,e_w114661587-380,e_w1158716725,e_w118987056-380,e_w143585004-380,e_w145665799-380,e_w145665862-380,e_w146791215-380,e_w149997403-380,e_w155590373-380,e_w157912118-380,e_w158739183-380,e_w172302572-380,e_w199675964-380,e_w203225567,e_w255011550-380,e_w303915533-380,e_w338753171-380,e_w36873258-380,e_w409439916-380,e_w411026199-380,e_w414663585-380,e_w416989699-380,e_w418902800-380,e_w432729521-380,e_w491424937-380,e_w491424937-400,e_w58992998-380,e_w591027058-380,e_w59219335-380,e_w59462715-380,e_w60725875-380,e_w60913666-380,e_w60919237-380,e_w72570378-380,e_w72570474-380,e_w743450089-380,e_w74943205-380,e_w81929591-380,e_w82759380-380,e_w82762493-380,e_w82767145-380,e_w83872215-380</t>
   </si>
 </sst>
 </file>
@@ -3187,7 +3193,7 @@
       </c>
       <c r="L27" t="str">
         <f>$V$28</f>
-        <v>ELC</v>
+        <v>e_IT10-380,e_IT156-380,e_IT157-380,e_IT158-380,e_IT159-380,e_IT21-380,e_IT42-380,e_IT7-380,e_IT8-380,e_IT9-380,e_IT90-400,e_IT93-380,e_w100113593-380,e_w100407576-380,e_w103381531-380,e_w103653592-380,e_w105757794-380,e_w109588422-380,e_w109756016-380,e_w109993642-380,e_w109997676-380,e_w110138220-380,e_w1103579629-380,e_w110660048-380,e_w1117128898-380,e_w114661587-380,e_w1158716725,e_w118987056-380,e_w143585004-380,e_w145665799-380,e_w145665862-380,e_w146791215-380,e_w149997403-380,e_w155590373-380,e_w157912118-380,e_w158739183-380,e_w172302572-380,e_w199675964-380,e_w203225567,e_w255011550-380,e_w303915533-380,e_w338753171-380,e_w36873258-380,e_w409439916-380,e_w411026199-380,e_w414663585-380,e_w416989699-380,e_w418902800-380,e_w432729521-380,e_w491424937-380,e_w491424937-400,e_w58992998-380,e_w591027058-380,e_w59219335-380,e_w59462715-380,e_w60725875-380,e_w60913666-380,e_w60919237-380,e_w72570378-380,e_w72570474-380,e_w743450089-380,e_w74943205-380,e_w81929591-380,e_w82759380-380,e_w82762493-380,e_w82767145-380,e_w83872215-380</v>
       </c>
       <c r="P27">
         <v>0</v>
@@ -3209,7 +3215,7 @@
       </c>
       <c r="K28" t="str">
         <f>$V$28</f>
-        <v>ELC</v>
+        <v>e_IT10-380,e_IT156-380,e_IT157-380,e_IT158-380,e_IT159-380,e_IT21-380,e_IT42-380,e_IT7-380,e_IT8-380,e_IT9-380,e_IT90-400,e_IT93-380,e_w100113593-380,e_w100407576-380,e_w103381531-380,e_w103653592-380,e_w105757794-380,e_w109588422-380,e_w109756016-380,e_w109993642-380,e_w109997676-380,e_w110138220-380,e_w1103579629-380,e_w110660048-380,e_w1117128898-380,e_w114661587-380,e_w1158716725,e_w118987056-380,e_w143585004-380,e_w145665799-380,e_w145665862-380,e_w146791215-380,e_w149997403-380,e_w155590373-380,e_w157912118-380,e_w158739183-380,e_w172302572-380,e_w199675964-380,e_w203225567,e_w255011550-380,e_w303915533-380,e_w338753171-380,e_w36873258-380,e_w409439916-380,e_w411026199-380,e_w414663585-380,e_w416989699-380,e_w418902800-380,e_w432729521-380,e_w491424937-380,e_w491424937-400,e_w58992998-380,e_w591027058-380,e_w59219335-380,e_w59462715-380,e_w60725875-380,e_w60913666-380,e_w60919237-380,e_w72570378-380,e_w72570474-380,e_w743450089-380,e_w74943205-380,e_w81929591-380,e_w82759380-380,e_w82762493-380,e_w82767145-380,e_w83872215-380</v>
       </c>
       <c r="P28">
         <v>0</v>
@@ -3224,7 +3230,7 @@
         <v>50</v>
       </c>
       <c r="V28" s="147" t="s">
-        <v>19</v>
+        <v>390</v>
       </c>
     </row>
   </sheetData>
@@ -4701,9 +4707,8 @@
     <row r="8" spans="2:25" ht="17.649999999999999">
       <c r="B8" s="20"/>
       <c r="E8" s="26"/>
-      <c r="F8" t="str">
-        <f>C5</f>
-        <v>ELC</v>
+      <c r="F8" t="s">
+        <v>163</v>
       </c>
       <c r="G8" t="str">
         <f>E7</f>
@@ -6026,62 +6031,62 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AEA11AE-74FD-454F-A049-805E4E5C4961}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0BBB19F-2A30-4639-A8ED-E1B6EAFA062D}">
   <dimension ref="B9:M34"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="9" spans="2:13">
       <c r="B9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J9" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="10" spans="2:13">
       <c r="B10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D10" t="s">
+        <v>167</v>
+      </c>
+      <c r="E10" t="s">
+        <v>168</v>
+      </c>
+      <c r="F10" t="s">
+        <v>169</v>
+      </c>
+      <c r="G10" t="s">
+        <v>170</v>
+      </c>
+      <c r="H10" t="s">
+        <v>171</v>
+      </c>
+      <c r="J10" t="s">
         <v>166</v>
       </c>
-      <c r="E10" t="s">
-        <v>167</v>
-      </c>
-      <c r="F10" t="s">
-        <v>168</v>
-      </c>
-      <c r="G10" t="s">
-        <v>169</v>
-      </c>
-      <c r="H10" t="s">
-        <v>170</v>
-      </c>
-      <c r="J10" t="s">
-        <v>165</v>
-      </c>
       <c r="K10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="L10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="M10" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="11" spans="2:13">
       <c r="B11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E11" t="s">
         <v>10</v>
@@ -6090,16 +6095,16 @@
         <v>21</v>
       </c>
       <c r="G11" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="K11" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="L11">
         <v>4.8756887454995406</v>
@@ -6110,13 +6115,13 @@
     </row>
     <row r="12" spans="2:13">
       <c r="B12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C12" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D12" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E12" t="s">
         <v>10</v>
@@ -6125,16 +6130,16 @@
         <v>21</v>
       </c>
       <c r="G12" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J12" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K12" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="L12">
         <v>24.363080093927088</v>
@@ -6145,13 +6150,13 @@
     </row>
     <row r="13" spans="2:13">
       <c r="B13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C13" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D13" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E13" t="s">
         <v>10</v>
@@ -6160,16 +6165,16 @@
         <v>21</v>
       </c>
       <c r="G13" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H13" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J13" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K13" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="L13">
         <v>0.11523048421685045</v>
@@ -6180,13 +6185,13 @@
     </row>
     <row r="14" spans="2:13">
       <c r="B14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C14" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D14" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E14" t="s">
         <v>10</v>
@@ -6195,16 +6200,16 @@
         <v>21</v>
       </c>
       <c r="G14" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H14" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J14" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K14" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="L14">
         <v>12.370290287147224</v>
@@ -6215,13 +6220,13 @@
     </row>
     <row r="15" spans="2:13">
       <c r="B15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C15" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D15" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E15" t="s">
         <v>10</v>
@@ -6230,16 +6235,16 @@
         <v>21</v>
       </c>
       <c r="G15" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H15" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J15" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K15" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="L15">
         <v>9.4040580871581625E-2</v>
@@ -6250,13 +6255,13 @@
     </row>
     <row r="16" spans="2:13">
       <c r="B16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C16" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D16" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E16" t="s">
         <v>10</v>
@@ -6265,16 +6270,16 @@
         <v>21</v>
       </c>
       <c r="G16" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H16" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J16" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="K16" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="L16">
         <v>5.8282611827233533</v>
@@ -6285,13 +6290,13 @@
     </row>
     <row r="17" spans="2:13">
       <c r="B17" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D17" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E17" t="s">
         <v>10</v>
@@ -6300,16 +6305,16 @@
         <v>21</v>
       </c>
       <c r="G17" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H17" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="K17" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="L17">
         <v>44.98318285576746</v>
@@ -6320,13 +6325,13 @@
     </row>
     <row r="18" spans="2:13">
       <c r="B18" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C18" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D18" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E18" t="s">
         <v>10</v>
@@ -6335,16 +6340,16 @@
         <v>21</v>
       </c>
       <c r="G18" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H18" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J18" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="K18" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="L18">
         <v>2.7793460957217331</v>
@@ -6355,13 +6360,13 @@
     </row>
     <row r="19" spans="2:13">
       <c r="B19" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C19" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D19" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E19" t="s">
         <v>10</v>
@@ -6370,16 +6375,16 @@
         <v>21</v>
       </c>
       <c r="G19" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H19" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J19" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K19" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="L19">
         <v>6.641615412118532</v>
@@ -6390,13 +6395,13 @@
     </row>
     <row r="20" spans="2:13">
       <c r="B20" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C20" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D20" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E20" t="s">
         <v>10</v>
@@ -6405,16 +6410,16 @@
         <v>21</v>
       </c>
       <c r="G20" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H20" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J20" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="K20" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L20">
         <v>10.705533259062522</v>
@@ -6425,13 +6430,13 @@
     </row>
     <row r="21" spans="2:13">
       <c r="B21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C21" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D21" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E21" t="s">
         <v>10</v>
@@ -6440,16 +6445,16 @@
         <v>21</v>
       </c>
       <c r="G21" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H21" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J21" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="K21" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="L21">
         <v>7.8151942553314413</v>
@@ -6460,13 +6465,13 @@
     </row>
     <row r="22" spans="2:13">
       <c r="B22" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C22" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D22" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E22" t="s">
         <v>10</v>
@@ -6475,16 +6480,16 @@
         <v>21</v>
       </c>
       <c r="G22" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H22" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J22" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="K22" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="L22">
         <v>3.787245058440587</v>
@@ -6495,13 +6500,13 @@
     </row>
     <row r="23" spans="2:13">
       <c r="B23" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C23" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D23" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E23" t="s">
         <v>10</v>
@@ -6510,16 +6515,16 @@
         <v>21</v>
       </c>
       <c r="G23" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H23" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J23" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="K23" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="L23">
         <v>11.035354442158566</v>
@@ -6530,13 +6535,13 @@
     </row>
     <row r="24" spans="2:13">
       <c r="B24" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C24" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D24" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E24" t="s">
         <v>10</v>
@@ -6545,16 +6550,16 @@
         <v>21</v>
       </c>
       <c r="G24" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H24" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J24" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="K24" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="L24">
         <v>5.7113903390121514</v>
@@ -6565,13 +6570,13 @@
     </row>
     <row r="25" spans="2:13">
       <c r="B25" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C25" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D25" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E25" t="s">
         <v>10</v>
@@ -6580,16 +6585,16 @@
         <v>21</v>
       </c>
       <c r="G25" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H25" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J25" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="K25" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="L25">
         <v>9.0662172460897033</v>
@@ -6600,13 +6605,13 @@
     </row>
     <row r="26" spans="2:13">
       <c r="B26" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C26" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D26" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E26" t="s">
         <v>10</v>
@@ -6615,16 +6620,16 @@
         <v>21</v>
       </c>
       <c r="G26" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H26" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J26" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="K26" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="L26">
         <v>19.420870985373586</v>
@@ -6635,13 +6640,13 @@
     </row>
     <row r="27" spans="2:13">
       <c r="B27" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C27" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D27" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E27" t="s">
         <v>10</v>
@@ -6650,16 +6655,16 @@
         <v>21</v>
       </c>
       <c r="G27" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H27" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J27" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="K27" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="L27">
         <v>7.539956732039311</v>
@@ -6670,13 +6675,13 @@
     </row>
     <row r="28" spans="2:13">
       <c r="B28" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C28" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D28" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E28" t="s">
         <v>10</v>
@@ -6685,16 +6690,16 @@
         <v>21</v>
       </c>
       <c r="G28" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H28" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J28" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K28" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="L28">
         <v>11.33028486424983</v>
@@ -6705,13 +6710,13 @@
     </row>
     <row r="29" spans="2:13">
       <c r="B29" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C29" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D29" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E29" t="s">
         <v>10</v>
@@ -6720,16 +6725,16 @@
         <v>21</v>
       </c>
       <c r="G29" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H29" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J29" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="K29" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="L29">
         <v>9.520512324694101</v>
@@ -6740,13 +6745,13 @@
     </row>
     <row r="30" spans="2:13">
       <c r="B30" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C30" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D30" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E30" t="s">
         <v>10</v>
@@ -6755,16 +6760,16 @@
         <v>21</v>
       </c>
       <c r="G30" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H30" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J30" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="K30" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="L30">
         <v>15.622210660715986</v>
@@ -6775,13 +6780,13 @@
     </row>
     <row r="31" spans="2:13">
       <c r="B31" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C31" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D31" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E31" t="s">
         <v>10</v>
@@ -6790,16 +6795,16 @@
         <v>21</v>
       </c>
       <c r="G31" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H31" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J31" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="K31" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="L31">
         <v>12.374405982824484</v>
@@ -6810,13 +6815,13 @@
     </row>
     <row r="32" spans="2:13">
       <c r="B32" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C32" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D32" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E32" t="s">
         <v>10</v>
@@ -6825,16 +6830,16 @@
         <v>21</v>
       </c>
       <c r="G32" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H32" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J32" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="K32" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="L32">
         <v>19.338901625217922</v>
@@ -6845,13 +6850,13 @@
     </row>
     <row r="33" spans="2:13">
       <c r="B33" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C33" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D33" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E33" t="s">
         <v>10</v>
@@ -6860,16 +6865,16 @@
         <v>21</v>
       </c>
       <c r="G33" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H33" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J33" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="K33" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="L33">
         <v>7.6634505148876118</v>
@@ -6880,13 +6885,13 @@
     </row>
     <row r="34" spans="2:13">
       <c r="B34" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C34" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D34" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E34" t="s">
         <v>10</v>
@@ -6895,16 +6900,16 @@
         <v>21</v>
       </c>
       <c r="G34" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H34" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J34" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="K34" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="L34">
         <v>8.1016831146845654</v>
@@ -6919,101 +6924,101 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64848B6E-95B5-499E-A155-0D07EBA48C92}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE44B0DA-F533-40CF-B981-EC76FC1F6DD3}">
   <dimension ref="B9:Z29"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="9" spans="2:26">
       <c r="B9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J9" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="O9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="W9" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="10" spans="2:26">
       <c r="B10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C10" t="s">
+        <v>166</v>
+      </c>
+      <c r="D10" t="s">
+        <v>167</v>
+      </c>
+      <c r="E10" t="s">
+        <v>168</v>
+      </c>
+      <c r="F10" t="s">
+        <v>169</v>
+      </c>
+      <c r="G10" t="s">
+        <v>170</v>
+      </c>
+      <c r="H10" t="s">
+        <v>171</v>
+      </c>
+      <c r="J10" t="s">
+        <v>166</v>
+      </c>
+      <c r="K10" t="s">
+        <v>224</v>
+      </c>
+      <c r="L10" t="s">
+        <v>225</v>
+      </c>
+      <c r="M10" t="s">
+        <v>226</v>
+      </c>
+      <c r="O10" t="s">
         <v>165</v>
       </c>
-      <c r="D10" t="s">
+      <c r="P10" t="s">
         <v>166</v>
       </c>
-      <c r="E10" t="s">
+      <c r="Q10" t="s">
         <v>167</v>
       </c>
-      <c r="F10" t="s">
+      <c r="R10" t="s">
         <v>168</v>
       </c>
-      <c r="G10" t="s">
+      <c r="S10" t="s">
         <v>169</v>
       </c>
-      <c r="H10" t="s">
+      <c r="T10" t="s">
         <v>170</v>
       </c>
-      <c r="J10" t="s">
-        <v>165</v>
-      </c>
-      <c r="K10" t="s">
-        <v>223</v>
-      </c>
-      <c r="L10" t="s">
+      <c r="U10" t="s">
+        <v>171</v>
+      </c>
+      <c r="W10" t="s">
+        <v>166</v>
+      </c>
+      <c r="X10" t="s">
         <v>224</v>
       </c>
-      <c r="M10" t="s">
+      <c r="Y10" t="s">
         <v>225</v>
       </c>
-      <c r="O10" t="s">
-        <v>164</v>
-      </c>
-      <c r="P10" t="s">
-        <v>165</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>166</v>
-      </c>
-      <c r="R10" t="s">
-        <v>167</v>
-      </c>
-      <c r="S10" t="s">
-        <v>168</v>
-      </c>
-      <c r="T10" t="s">
-        <v>169</v>
-      </c>
-      <c r="U10" t="s">
-        <v>170</v>
-      </c>
-      <c r="W10" t="s">
-        <v>165</v>
-      </c>
-      <c r="X10" t="s">
-        <v>223</v>
-      </c>
-      <c r="Y10" t="s">
-        <v>224</v>
-      </c>
       <c r="Z10" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="11" spans="2:26">
       <c r="B11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C11" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D11" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E11" t="s">
         <v>10</v>
@@ -7022,16 +7027,16 @@
         <v>21</v>
       </c>
       <c r="G11" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J11" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="K11" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="L11">
         <v>7.7363165779076795</v>
@@ -7040,13 +7045,13 @@
         <v>0.1067814682163853</v>
       </c>
       <c r="O11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P11" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="Q11" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="R11" t="s">
         <v>10</v>
@@ -7055,16 +7060,16 @@
         <v>21</v>
       </c>
       <c r="T11" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W11" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="X11" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="Y11">
         <v>39.450749999999999</v>
@@ -7075,13 +7080,13 @@
     </row>
     <row r="12" spans="2:26">
       <c r="B12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C12" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D12" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E12" t="s">
         <v>10</v>
@@ -7090,16 +7095,16 @@
         <v>21</v>
       </c>
       <c r="G12" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J12" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="K12" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="L12">
         <v>2.3427652611420688</v>
@@ -7108,13 +7113,13 @@
         <v>0.24330473042687509</v>
       </c>
       <c r="O12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P12" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="Q12" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="R12" t="s">
         <v>10</v>
@@ -7123,16 +7128,16 @@
         <v>21</v>
       </c>
       <c r="T12" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U12" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W12" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="X12" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="Y12">
         <v>10.7745</v>
@@ -7143,13 +7148,13 @@
     </row>
     <row r="13" spans="2:26">
       <c r="B13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C13" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D13" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E13" t="s">
         <v>10</v>
@@ -7158,16 +7163,16 @@
         <v>21</v>
       </c>
       <c r="G13" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H13" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J13" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="K13" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="L13">
         <v>21.492626448742886</v>
@@ -7176,13 +7181,13 @@
         <v>0.1659864827149567</v>
       </c>
       <c r="O13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P13" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="Q13" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="R13" t="s">
         <v>10</v>
@@ -7191,16 +7196,16 @@
         <v>21</v>
       </c>
       <c r="T13" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U13" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W13" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="X13" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="Y13">
         <v>38.600250000000003</v>
@@ -7211,13 +7216,13 @@
     </row>
     <row r="14" spans="2:26">
       <c r="B14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C14" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D14" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E14" t="s">
         <v>10</v>
@@ -7226,16 +7231,16 @@
         <v>21</v>
       </c>
       <c r="G14" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H14" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J14" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="K14" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="L14">
         <v>6.3986137173550848</v>
@@ -7244,13 +7249,13 @@
         <v>0.12695115959174291</v>
       </c>
       <c r="O14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P14" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="Q14" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="R14" t="s">
         <v>10</v>
@@ -7259,16 +7264,16 @@
         <v>21</v>
       </c>
       <c r="T14" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U14" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W14" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="X14" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="Y14">
         <v>4.0402500000000003</v>
@@ -7279,13 +7284,13 @@
     </row>
     <row r="15" spans="2:26">
       <c r="B15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C15" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D15" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E15" t="s">
         <v>10</v>
@@ -7294,16 +7299,16 @@
         <v>21</v>
       </c>
       <c r="G15" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H15" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J15" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="K15" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="L15">
         <v>4.0537250245901548</v>
@@ -7312,13 +7317,13 @@
         <v>0.1156289487533637</v>
       </c>
       <c r="O15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P15" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="Q15" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="R15" t="s">
         <v>10</v>
@@ -7327,16 +7332,16 @@
         <v>21</v>
       </c>
       <c r="T15" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U15" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W15" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="X15" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="Y15">
         <v>39.321750000000002</v>
@@ -7347,13 +7352,13 @@
     </row>
     <row r="16" spans="2:26">
       <c r="B16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C16" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D16" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E16" t="s">
         <v>10</v>
@@ -7362,16 +7367,16 @@
         <v>21</v>
       </c>
       <c r="G16" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H16" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J16" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="K16" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="L16">
         <v>9.6185391844194168</v>
@@ -7380,13 +7385,13 @@
         <v>8.8659780776036604E-2</v>
       </c>
       <c r="O16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P16" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="Q16" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="R16" t="s">
         <v>10</v>
@@ -7395,16 +7400,16 @@
         <v>21</v>
       </c>
       <c r="T16" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U16" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W16" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="X16" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="Y16">
         <v>12.592499999999999</v>
@@ -7415,13 +7420,13 @@
     </row>
     <row r="17" spans="2:26">
       <c r="B17" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C17" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D17" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E17" t="s">
         <v>10</v>
@@ -7430,16 +7435,16 @@
         <v>21</v>
       </c>
       <c r="G17" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H17" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J17" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="K17" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="L17">
         <v>20.992062966824207</v>
@@ -7448,13 +7453,13 @@
         <v>0.113712621553391</v>
       </c>
       <c r="O17" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P17" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="Q17" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="R17" t="s">
         <v>10</v>
@@ -7463,16 +7468,16 @@
         <v>21</v>
       </c>
       <c r="T17" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U17" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W17" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="X17" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="Y17">
         <v>15.871499999999999</v>
@@ -7483,13 +7488,13 @@
     </row>
     <row r="18" spans="2:26">
       <c r="B18" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C18" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D18" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E18" t="s">
         <v>10</v>
@@ -7498,16 +7503,16 @@
         <v>21</v>
       </c>
       <c r="G18" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H18" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J18" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="K18" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="L18">
         <v>4.7225970155809494</v>
@@ -7516,13 +7521,13 @@
         <v>0.11595533842419591</v>
       </c>
       <c r="O18" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P18" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="Q18" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="R18" t="s">
         <v>10</v>
@@ -7531,16 +7536,16 @@
         <v>21</v>
       </c>
       <c r="T18" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U18" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W18" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="X18" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="Y18">
         <v>19.04175</v>
@@ -7551,13 +7556,13 @@
     </row>
     <row r="19" spans="2:26">
       <c r="B19" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C19" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D19" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E19" t="s">
         <v>10</v>
@@ -7566,16 +7571,16 @@
         <v>21</v>
       </c>
       <c r="G19" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H19" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J19" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="K19" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="L19">
         <v>9.0836490896593176</v>
@@ -7584,13 +7589,13 @@
         <v>0.13201736314252621</v>
       </c>
       <c r="O19" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P19" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="Q19" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="R19" t="s">
         <v>10</v>
@@ -7599,16 +7604,16 @@
         <v>21</v>
       </c>
       <c r="T19" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U19" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W19" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="X19" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="Y19">
         <v>28.344000000000001</v>
@@ -7619,13 +7624,13 @@
     </row>
     <row r="20" spans="2:26">
       <c r="B20" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C20" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D20" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E20" t="s">
         <v>10</v>
@@ -7634,16 +7639,16 @@
         <v>21</v>
       </c>
       <c r="G20" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H20" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J20" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="K20" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="L20">
         <v>10.618766499150132</v>
@@ -7652,13 +7657,13 @@
         <v>0.1639958713693849</v>
       </c>
       <c r="O20" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P20" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="Q20" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="R20" t="s">
         <v>10</v>
@@ -7667,16 +7672,16 @@
         <v>21</v>
       </c>
       <c r="T20" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U20" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W20" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="X20" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="Y20">
         <v>14.163</v>
@@ -7687,13 +7692,13 @@
     </row>
     <row r="21" spans="2:26">
       <c r="B21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C21" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D21" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E21" t="s">
         <v>10</v>
@@ -7702,16 +7707,16 @@
         <v>21</v>
       </c>
       <c r="G21" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H21" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J21" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="K21" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="L21">
         <v>37.276481001553563</v>
@@ -7720,13 +7725,13 @@
         <v>0.20831242550980769</v>
       </c>
       <c r="O21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P21" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="Q21" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="R21" t="s">
         <v>10</v>
@@ -7735,16 +7740,16 @@
         <v>21</v>
       </c>
       <c r="T21" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U21" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W21" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="X21" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="Y21">
         <v>2.0775000000000001</v>
@@ -7755,13 +7760,13 @@
     </row>
     <row r="22" spans="2:26">
       <c r="B22" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C22" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D22" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E22" t="s">
         <v>10</v>
@@ -7770,16 +7775,16 @@
         <v>21</v>
       </c>
       <c r="G22" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H22" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J22" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="K22" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="L22">
         <v>20.90644030096918</v>
@@ -7788,13 +7793,13 @@
         <v>0.1089207512006329</v>
       </c>
       <c r="O22" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P22" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="Q22" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="R22" t="s">
         <v>10</v>
@@ -7803,16 +7808,16 @@
         <v>21</v>
       </c>
       <c r="T22" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U22" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W22" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="X22" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="Y22">
         <v>9.2415000000000003</v>
@@ -7823,13 +7828,13 @@
     </row>
     <row r="23" spans="2:26">
       <c r="B23" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C23" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D23" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E23" t="s">
         <v>10</v>
@@ -7838,16 +7843,16 @@
         <v>21</v>
       </c>
       <c r="G23" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H23" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J23" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="K23" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="L23">
         <v>1.24293744829465</v>
@@ -7856,13 +7861,13 @@
         <v>9.4018179307857899E-2</v>
       </c>
       <c r="O23" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P23" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="Q23" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="R23" t="s">
         <v>10</v>
@@ -7871,16 +7876,16 @@
         <v>21</v>
       </c>
       <c r="T23" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U23" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W23" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="X23" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="Y23">
         <v>0.97650000000000003</v>
@@ -7891,13 +7896,13 @@
     </row>
     <row r="24" spans="2:26">
       <c r="B24" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C24" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D24" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E24" t="s">
         <v>10</v>
@@ -7906,16 +7911,16 @@
         <v>21</v>
       </c>
       <c r="G24" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H24" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J24" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="K24" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="L24">
         <v>3.655060122103603</v>
@@ -7924,13 +7929,13 @@
         <v>0.14311265140153179</v>
       </c>
       <c r="O24" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P24" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="Q24" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="R24" t="s">
         <v>10</v>
@@ -7939,16 +7944,16 @@
         <v>21</v>
       </c>
       <c r="T24" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U24" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W24" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="X24" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="Y24">
         <v>6.8857499999999998</v>
@@ -7959,13 +7964,13 @@
     </row>
     <row r="25" spans="2:26">
       <c r="B25" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C25" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D25" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E25" t="s">
         <v>10</v>
@@ -7974,16 +7979,16 @@
         <v>21</v>
       </c>
       <c r="G25" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H25" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J25" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="K25" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="L25">
         <v>48.450394178145253</v>
@@ -7992,13 +7997,13 @@
         <v>0.2433164831628466</v>
       </c>
       <c r="O25" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P25" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="Q25" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="R25" t="s">
         <v>10</v>
@@ -8007,16 +8012,16 @@
         <v>21</v>
       </c>
       <c r="T25" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U25" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W25" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="X25" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="Y25">
         <v>71.778000000000006</v>
@@ -8027,13 +8032,13 @@
     </row>
     <row r="26" spans="2:26">
       <c r="B26" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C26" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D26" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E26" t="s">
         <v>10</v>
@@ -8042,16 +8047,16 @@
         <v>21</v>
       </c>
       <c r="G26" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H26" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J26" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="K26" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="L26">
         <v>19.948651692996549</v>
@@ -8060,13 +8065,13 @@
         <v>0.26469960967055511</v>
       </c>
       <c r="O26" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P26" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="Q26" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="R26" t="s">
         <v>10</v>
@@ -8075,16 +8080,16 @@
         <v>21</v>
       </c>
       <c r="T26" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U26" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W26" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="X26" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="Y26">
         <v>40.861499999999999</v>
@@ -8095,13 +8100,13 @@
     </row>
     <row r="27" spans="2:26">
       <c r="B27" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C27" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D27" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E27" t="s">
         <v>10</v>
@@ -8110,16 +8115,16 @@
         <v>21</v>
       </c>
       <c r="G27" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H27" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J27" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="K27" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L27">
         <v>23.13749613808001</v>
@@ -8128,13 +8133,13 @@
         <v>0.13108526943306451</v>
       </c>
       <c r="O27" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P27" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="Q27" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="R27" t="s">
         <v>10</v>
@@ -8143,16 +8148,16 @@
         <v>21</v>
       </c>
       <c r="T27" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U27" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W27" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="X27" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="Y27">
         <v>53.390250000000002</v>
@@ -8163,13 +8168,13 @@
     </row>
     <row r="28" spans="2:26">
       <c r="B28" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C28" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D28" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E28" t="s">
         <v>10</v>
@@ -8178,16 +8183,16 @@
         <v>21</v>
       </c>
       <c r="G28" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H28" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J28" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="K28" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="L28">
         <v>6.7463178806119855</v>
@@ -8196,13 +8201,13 @@
         <v>0.13784704004674381</v>
       </c>
       <c r="O28" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P28" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="Q28" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="R28" t="s">
         <v>10</v>
@@ -8211,16 +8216,16 @@
         <v>21</v>
       </c>
       <c r="T28" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U28" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W28" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="X28" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="Y28">
         <v>49.423499999999997</v>
@@ -8231,13 +8236,13 @@
     </row>
     <row r="29" spans="2:26">
       <c r="B29" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C29" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D29" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E29" t="s">
         <v>10</v>
@@ -8246,16 +8251,16 @@
         <v>21</v>
       </c>
       <c r="G29" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H29" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J29" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="K29" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="L29">
         <v>9.7794224100622564</v>
@@ -8264,13 +8269,13 @@
         <v>0.1332508824588724</v>
       </c>
       <c r="O29" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P29" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="Q29" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="R29" t="s">
         <v>10</v>
@@ -8279,16 +8284,16 @@
         <v>21</v>
       </c>
       <c r="T29" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U29" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="W29" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="X29" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="Y29">
         <v>48.613500000000002</v>
@@ -8303,27 +8308,27 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74610678-2E1E-4A97-AFF7-27BC399EDA63}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A19EE99-7250-4944-BD16-5B2C2C03B31E}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="9" spans="2:16">
       <c r="B9" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="J9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="10" spans="2:16">
       <c r="B10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C10" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="D10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E10">
         <v>2023</v>
@@ -8338,30 +8343,30 @@
         <v>54</v>
       </c>
       <c r="J10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="L10" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="M10" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="N10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="O10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="P10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="11" spans="2:16">
       <c r="B11" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C11" t="s">
         <v>31</v>
@@ -8382,10 +8387,10 @@
         <v>146</v>
       </c>
       <c r="J11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K11" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="M11" t="s">
         <v>10</v>
@@ -8394,15 +8399,15 @@
         <v>21</v>
       </c>
       <c r="O11" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="P11" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="12" spans="2:16">
       <c r="B12" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C12" t="s">
         <v>31</v>
@@ -8420,13 +8425,13 @@
         <v>0.60000000000000009</v>
       </c>
       <c r="H12" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="J12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K12" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="M12" t="s">
         <v>10</v>
@@ -8435,15 +8440,15 @@
         <v>21</v>
       </c>
       <c r="O12" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="P12" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="13" spans="2:16">
       <c r="B13" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C13" t="s">
         <v>31</v>
@@ -8461,13 +8466,13 @@
         <v>5100</v>
       </c>
       <c r="H13" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="J13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K13" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="M13" t="s">
         <v>10</v>
@@ -8476,15 +8481,15 @@
         <v>21</v>
       </c>
       <c r="O13" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="P13" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="14" spans="2:16">
       <c r="B14" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C14" t="s">
         <v>31</v>
@@ -8502,13 +8507,13 @@
         <v>175</v>
       </c>
       <c r="H14" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="J14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K14" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="M14" t="s">
         <v>10</v>
@@ -8517,15 +8522,15 @@
         <v>21</v>
       </c>
       <c r="O14" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="P14" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="15" spans="2:16">
       <c r="B15" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C15" t="s">
         <v>31</v>
@@ -8543,13 +8548,13 @@
         <v>3</v>
       </c>
       <c r="H15" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="J15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K15" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="M15" t="s">
         <v>10</v>
@@ -8558,15 +8563,15 @@
         <v>21</v>
       </c>
       <c r="O15" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="P15" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="16" spans="2:16">
       <c r="B16" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C16" t="s">
         <v>31</v>
@@ -8587,10 +8592,10 @@
         <v>146</v>
       </c>
       <c r="J16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K16" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="M16" t="s">
         <v>10</v>
@@ -8599,15 +8604,15 @@
         <v>21</v>
       </c>
       <c r="O16" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="P16" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="17" spans="2:16">
       <c r="B17" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C17" t="s">
         <v>31</v>
@@ -8625,13 +8630,13 @@
         <v>0.60000000000000009</v>
       </c>
       <c r="H17" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="J17" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K17" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="M17" t="s">
         <v>10</v>
@@ -8640,15 +8645,15 @@
         <v>21</v>
       </c>
       <c r="O17" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="P17" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="18" spans="2:16">
       <c r="B18" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C18" t="s">
         <v>31</v>
@@ -8666,13 +8671,13 @@
         <v>2300</v>
       </c>
       <c r="H18" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="J18" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K18" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="M18" t="s">
         <v>10</v>
@@ -8681,15 +8686,15 @@
         <v>21</v>
       </c>
       <c r="O18" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="P18" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="19" spans="2:16">
       <c r="B19" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C19" t="s">
         <v>31</v>
@@ -8707,13 +8712,13 @@
         <v>80</v>
       </c>
       <c r="H19" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="J19" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K19" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="M19" t="s">
         <v>10</v>
@@ -8722,15 +8727,15 @@
         <v>21</v>
       </c>
       <c r="O19" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="P19" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="20" spans="2:16">
       <c r="B20" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C20" t="s">
         <v>31</v>
@@ -8748,13 +8753,13 @@
         <v>3</v>
       </c>
       <c r="H20" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="J20" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K20" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="M20" t="s">
         <v>10</v>
@@ -8763,15 +8768,15 @@
         <v>21</v>
       </c>
       <c r="O20" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="P20" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="21" spans="2:16">
       <c r="B21" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C21" t="s">
         <v>33</v>
@@ -8792,10 +8797,10 @@
         <v>146</v>
       </c>
       <c r="J21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K21" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="M21" t="s">
         <v>10</v>
@@ -8804,15 +8809,15 @@
         <v>21</v>
       </c>
       <c r="O21" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="P21" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="22" spans="2:16">
       <c r="B22" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C22" t="s">
         <v>33</v>
@@ -8830,13 +8835,13 @@
         <v>1000</v>
       </c>
       <c r="H22" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="J22" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K22" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="M22" t="s">
         <v>10</v>
@@ -8845,15 +8850,15 @@
         <v>21</v>
       </c>
       <c r="O22" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="P22" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="23" spans="2:16">
       <c r="B23" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C23" t="s">
         <v>33</v>
@@ -8871,13 +8876,13 @@
         <v>25</v>
       </c>
       <c r="H23" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="J23" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K23" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="M23" t="s">
         <v>10</v>
@@ -8886,15 +8891,15 @@
         <v>21</v>
       </c>
       <c r="O23" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="P23" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="24" spans="2:16">
       <c r="B24" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C24" t="s">
         <v>33</v>
@@ -8915,10 +8920,10 @@
         <v>146</v>
       </c>
       <c r="J24" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K24" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="M24" t="s">
         <v>10</v>
@@ -8927,15 +8932,15 @@
         <v>21</v>
       </c>
       <c r="O24" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="P24" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="25" spans="2:16">
       <c r="B25" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C25" t="s">
         <v>33</v>
@@ -8953,13 +8958,13 @@
         <v>2400</v>
       </c>
       <c r="H25" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="J25" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K25" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="M25" t="s">
         <v>10</v>
@@ -8968,15 +8973,15 @@
         <v>21</v>
       </c>
       <c r="O25" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="P25" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="26" spans="2:16">
       <c r="B26" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C26" t="s">
         <v>33</v>
@@ -8994,13 +8999,13 @@
         <v>60</v>
       </c>
       <c r="H26" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="J26" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K26" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="M26" t="s">
         <v>10</v>
@@ -9009,15 +9014,15 @@
         <v>21</v>
       </c>
       <c r="O26" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="P26" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="27" spans="2:16">
       <c r="B27" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C27" t="s">
         <v>32</v>
@@ -9038,10 +9043,10 @@
         <v>146</v>
       </c>
       <c r="J27" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K27" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="M27" t="s">
         <v>10</v>
@@ -9050,15 +9055,15 @@
         <v>21</v>
       </c>
       <c r="O27" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="P27" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="28" spans="2:16">
       <c r="B28" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C28" t="s">
         <v>32</v>
@@ -9076,12 +9081,12 @@
         <v>4350</v>
       </c>
       <c r="H28" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="29" spans="2:16">
       <c r="B29" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C29" t="s">
         <v>32</v>
@@ -9099,12 +9104,12 @@
         <v>130</v>
       </c>
       <c r="H29" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="30" spans="2:16">
       <c r="B30" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C30" t="s">
         <v>33</v>
@@ -9127,7 +9132,7 @@
     </row>
     <row r="31" spans="2:16">
       <c r="B31" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C31" t="s">
         <v>33</v>
@@ -9145,12 +9150,12 @@
         <v>500</v>
       </c>
       <c r="H31" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="32" spans="2:16">
       <c r="B32" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C32" t="s">
         <v>33</v>
@@ -9168,12 +9173,12 @@
         <v>20</v>
       </c>
       <c r="H32" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="33" spans="2:8">
       <c r="B33" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C33" t="s">
         <v>28</v>
@@ -9196,7 +9201,7 @@
     </row>
     <row r="34" spans="2:8">
       <c r="B34" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C34" t="s">
         <v>28</v>
@@ -9214,12 +9219,12 @@
         <v>0.35000000000000003</v>
       </c>
       <c r="H34" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="35" spans="2:8">
       <c r="B35" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C35" t="s">
         <v>28</v>
@@ -9237,12 +9242,12 @@
         <v>2650</v>
       </c>
       <c r="H35" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="36" spans="2:8">
       <c r="B36" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C36" t="s">
         <v>28</v>
@@ -9260,12 +9265,12 @@
         <v>65</v>
       </c>
       <c r="H36" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="37" spans="2:8">
       <c r="B37" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C37" t="s">
         <v>28</v>
@@ -9283,12 +9288,12 @@
         <v>4</v>
       </c>
       <c r="H37" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
     </row>
     <row r="38" spans="2:8">
       <c r="B38" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C38" t="s">
         <v>33</v>
@@ -9311,7 +9316,7 @@
     </row>
     <row r="39" spans="2:8">
       <c r="B39" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C39" t="s">
         <v>33</v>
@@ -9329,12 +9334,12 @@
         <v>2300</v>
       </c>
       <c r="H39" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="40" spans="2:8">
       <c r="B40" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C40" t="s">
         <v>33</v>
@@ -9352,12 +9357,12 @@
         <v>80</v>
       </c>
       <c r="H40" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="41" spans="2:8">
       <c r="B41" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C41" t="s">
         <v>32</v>
@@ -9380,7 +9385,7 @@
     </row>
     <row r="42" spans="2:8">
       <c r="B42" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C42" t="s">
         <v>32</v>
@@ -9398,12 +9403,12 @@
         <v>5100</v>
       </c>
       <c r="H42" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="43" spans="2:8">
       <c r="B43" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C43" t="s">
         <v>32</v>
@@ -9421,12 +9426,12 @@
         <v>180</v>
       </c>
       <c r="H43" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="44" spans="2:8">
       <c r="B44" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C44" t="s">
         <v>36</v>
@@ -9449,7 +9454,7 @@
     </row>
     <row r="45" spans="2:8">
       <c r="B45" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C45" t="s">
         <v>36</v>
@@ -9467,12 +9472,12 @@
         <v>4500</v>
       </c>
       <c r="H45" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="46" spans="2:8">
       <c r="B46" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C46" t="s">
         <v>36</v>
@@ -9490,12 +9495,12 @@
         <v>160</v>
       </c>
       <c r="H46" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="47" spans="2:8">
       <c r="B47" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C47" t="s">
         <v>32</v>
@@ -9518,7 +9523,7 @@
     </row>
     <row r="48" spans="2:8">
       <c r="B48" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C48" t="s">
         <v>32</v>
@@ -9536,12 +9541,12 @@
         <v>5100</v>
       </c>
       <c r="H48" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="49" spans="2:8">
       <c r="B49" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C49" t="s">
         <v>32</v>
@@ -9559,12 +9564,12 @@
         <v>155</v>
       </c>
       <c r="H49" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="50" spans="2:8">
       <c r="B50" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C50" t="s">
         <v>27</v>
@@ -9587,7 +9592,7 @@
     </row>
     <row r="51" spans="2:8">
       <c r="B51" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C51" t="s">
         <v>27</v>
@@ -9605,12 +9610,12 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="H51" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="52" spans="2:8">
       <c r="B52" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C52" t="s">
         <v>27</v>
@@ -9628,12 +9633,12 @@
         <v>340</v>
       </c>
       <c r="H52" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="53" spans="2:8">
       <c r="B53" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C53" t="s">
         <v>27</v>
@@ -9651,12 +9656,12 @@
         <v>10</v>
       </c>
       <c r="H53" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="54" spans="2:8">
       <c r="B54" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C54" t="s">
         <v>27</v>
@@ -9674,12 +9679,12 @@
         <v>1.5</v>
       </c>
       <c r="H54" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
     </row>
     <row r="55" spans="2:8">
       <c r="B55" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C55" t="s">
         <v>32</v>
@@ -9702,7 +9707,7 @@
     </row>
     <row r="56" spans="2:8">
       <c r="B56" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C56" t="s">
         <v>32</v>
@@ -9720,12 +9725,12 @@
         <v>1700</v>
       </c>
       <c r="H56" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="57" spans="2:8">
       <c r="B57" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C57" t="s">
         <v>32</v>
@@ -9743,12 +9748,12 @@
         <v>45</v>
       </c>
       <c r="H57" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="58" spans="2:8">
       <c r="B58" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C58" t="s">
         <v>32</v>
@@ -9771,7 +9776,7 @@
     </row>
     <row r="59" spans="2:8">
       <c r="B59" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C59" t="s">
         <v>32</v>
@@ -9789,12 +9794,12 @@
         <v>2000</v>
       </c>
       <c r="H59" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="60" spans="2:8">
       <c r="B60" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C60" t="s">
         <v>32</v>
@@ -9812,12 +9817,12 @@
         <v>60</v>
       </c>
       <c r="H60" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="61" spans="2:8">
       <c r="B61" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C61" t="s">
         <v>32</v>
@@ -9840,7 +9845,7 @@
     </row>
     <row r="62" spans="2:8">
       <c r="B62" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C62" t="s">
         <v>32</v>
@@ -9858,12 +9863,12 @@
         <v>2200</v>
       </c>
       <c r="H62" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="63" spans="2:8">
       <c r="B63" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C63" t="s">
         <v>32</v>
@@ -9881,15 +9886,15 @@
         <v>65</v>
       </c>
       <c r="H63" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="64" spans="2:8">
       <c r="B64" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C64" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D64" t="s">
         <v>19</v>
@@ -9909,10 +9914,10 @@
     </row>
     <row r="65" spans="2:8">
       <c r="B65" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C65" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D65" t="s">
         <v>19</v>
@@ -9927,15 +9932,15 @@
         <v>0.56000000000000005</v>
       </c>
       <c r="H65" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="66" spans="2:8">
       <c r="B66" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C66" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D66" t="s">
         <v>19</v>
@@ -9950,15 +9955,15 @@
         <v>1660</v>
       </c>
       <c r="H66" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="67" spans="2:8">
       <c r="B67" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C67" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D67" t="s">
         <v>19</v>
@@ -9973,15 +9978,15 @@
         <v>40</v>
       </c>
       <c r="H67" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="68" spans="2:8">
       <c r="B68" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C68" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D68" t="s">
         <v>19</v>
@@ -9996,15 +10001,15 @@
         <v>3</v>
       </c>
       <c r="H68" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
     </row>
     <row r="69" spans="2:8">
       <c r="B69" t="s">
+        <v>387</v>
+      </c>
+      <c r="C69" t="s">
         <v>386</v>
-      </c>
-      <c r="C69" t="s">
-        <v>385</v>
       </c>
       <c r="D69" t="s">
         <v>19</v>
@@ -10024,10 +10029,10 @@
     </row>
     <row r="70" spans="2:8">
       <c r="B70" t="s">
+        <v>387</v>
+      </c>
+      <c r="C70" t="s">
         <v>386</v>
-      </c>
-      <c r="C70" t="s">
-        <v>385</v>
       </c>
       <c r="D70" t="s">
         <v>19</v>
@@ -10042,15 +10047,15 @@
         <v>0.3</v>
       </c>
       <c r="H70" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="71" spans="2:8">
       <c r="B71" t="s">
+        <v>387</v>
+      </c>
+      <c r="C71" t="s">
         <v>386</v>
-      </c>
-      <c r="C71" t="s">
-        <v>385</v>
       </c>
       <c r="D71" t="s">
         <v>19</v>
@@ -10065,15 +10070,15 @@
         <v>1490</v>
       </c>
       <c r="H71" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="72" spans="2:8">
       <c r="B72" t="s">
+        <v>387</v>
+      </c>
+      <c r="C72" t="s">
         <v>386</v>
-      </c>
-      <c r="C72" t="s">
-        <v>385</v>
       </c>
       <c r="D72" t="s">
         <v>19</v>
@@ -10088,15 +10093,15 @@
         <v>38</v>
       </c>
       <c r="H72" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="73" spans="2:8">
       <c r="B73" t="s">
+        <v>387</v>
+      </c>
+      <c r="C73" t="s">
         <v>386</v>
-      </c>
-      <c r="C73" t="s">
-        <v>385</v>
       </c>
       <c r="D73" t="s">
         <v>19</v>
@@ -10111,7 +10116,7 @@
         <v>1.5</v>
       </c>
       <c r="H73" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
     </row>
   </sheetData>

</xml_diff>